<commit_message>
Remove Daryl Loxham and Frankie Whitman from Team Realignment tab for consistency with Final Roster tab (both now 249 agents)
</commit_message>
<xml_diff>
--- a/2026-09-15/Team_Realignment_Review.xlsx
+++ b/2026-09-15/Team_Realignment_Review.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G252"/>
+  <dimension ref="A1:G250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5116,7 +5116,7 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Frankie Whitman (DBZ)</t>
+          <t>Reese Godfrey (DBZ)</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -5153,7 +5153,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Reese Godfrey (DBZ)</t>
+          <t>Teal Wainwright (DBZ)</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -5190,7 +5190,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Teal Wainwright (DBZ)</t>
+          <t>Spencer Baker (DBZ)</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -5227,7 +5227,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Spencer Baker (DBZ)</t>
+          <t>Darby Gearing (DBZ)</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -5264,7 +5264,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Darby Gearing (DBZ)</t>
+          <t>Rowan Redgrave (DBZ)</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -5301,7 +5301,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Rowan Redgrave (DBZ)</t>
+          <t>Tamsin Radford (DBZ)</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -5338,7 +5338,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Tamsin Radford (DBZ)</t>
+          <t>Ramsey Thomas (DBZ)</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -5375,7 +5375,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Ramsey Thomas (DBZ)</t>
+          <t>Sawyer Kempson (DBZ)</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -5412,12 +5412,12 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Sawyer Kempson (DBZ)</t>
+          <t>Harper Whitmore (DBZ)</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Riley Foster</t>
+          <t>Rory Sanderson</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -5449,17 +5449,17 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Harper Whitmore (DBZ)</t>
+          <t>Lindsay Wentworth (DBZ)</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Rory Sanderson</t>
+          <t>Frankie Baxter</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>Amari Ward</t>
+          <t>Sage Turner</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -5469,24 +5469,24 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>13:30-22:00</t>
+          <t>11:30-20:00</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>14:00-22:00</t>
+          <t>11:30-20:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>16</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Lindsay Wentworth (DBZ)</t>
+          <t>Kendall Ashcroft (DBZ)</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -5523,7 +5523,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Kendall Ashcroft (DBZ)</t>
+          <t>Leslie Walsingham (DBZ)</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -5560,7 +5560,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Leslie Walsingham (DBZ)</t>
+          <t>York Selwyn (DBZ)</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>York Selwyn (DBZ)</t>
+          <t>Sandy Lanchester (DBZ)</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -5634,7 +5634,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Sandy Lanchester (DBZ)</t>
+          <t>Callum Marlowe (DBZ)</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -5671,7 +5671,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Callum Marlowe (DBZ)</t>
+          <t>Rowan Ainsworth (DBZ)</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -5708,7 +5708,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Rowan Ainsworth (DBZ)</t>
+          <t>Kris Winstanley (DBZ)</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -5745,7 +5745,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Kris Winstanley (DBZ)</t>
+          <t>Lennox Darrow (DBZ)</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -5782,7 +5782,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Lennox Darrow (DBZ)</t>
+          <t>Nico Ellington (DBZ)</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -5819,7 +5819,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Nico Ellington (DBZ)</t>
+          <t>Jude Hartley (DBZ)</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -5854,46 +5854,46 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="inlineStr">
-        <is>
-          <t>Jude Hartley (DBZ)</t>
-        </is>
-      </c>
-      <c r="B147" s="2" t="inlineStr">
-        <is>
-          <t>Frankie Baxter</t>
-        </is>
-      </c>
-      <c r="C147" s="2" t="inlineStr">
-        <is>
-          <t>Sage Turner</t>
-        </is>
-      </c>
-      <c r="D147" s="2" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E147" s="2" t="inlineStr">
-        <is>
-          <t>11:30-20:00</t>
-        </is>
-      </c>
-      <c r="F147" s="2" t="inlineStr">
-        <is>
-          <t>11:30-20:00</t>
-        </is>
-      </c>
-      <c r="G147" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Jules Clarke (DBZ)</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Parker Jones</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Parker Jones</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>DBZ</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>07:00-15:30</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>07:00-15:00</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Jules Clarke (DBZ)</t>
+          <t>Cassidy Langley (DBZ)</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -5930,7 +5930,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Cassidy Langley (DBZ)</t>
+          <t>Arden Pritchard (DBZ)</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -5967,7 +5967,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Arden Pritchard (DBZ)</t>
+          <t>Marley Langley (DBZ)</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -6004,7 +6004,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Marley Langley (DBZ)</t>
+          <t>Frankie Middleton (DBZ)</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -6041,7 +6041,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Frankie Middleton (DBZ)</t>
+          <t>Nico Spencer (DBZ)</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -6078,7 +6078,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Nico Spencer (DBZ)</t>
+          <t>Devon Fairfax (DBZ)</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -6115,7 +6115,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Devon Fairfax (DBZ)</t>
+          <t>Gray Hollingsworth (DBZ)</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -6150,37 +6150,37 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>Gray Hollingsworth (DBZ)</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>Graylin Everard (DBZ)</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Morgan Shaw</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
         <is>
           <t>Parker Jones</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>Parker Jones</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr">
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>DBZ</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
         <is>
           <t>07:00-15:30</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr">
+      <c r="F155" s="2" t="inlineStr">
         <is>
           <t>07:00-15:00</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr">
+      <c r="G155" s="2" t="inlineStr">
         <is>
           <t>15</t>
         </is>
@@ -6189,7 +6189,7 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Graylin Everard (DBZ)</t>
+          <t>Harriet Bromley (DBZ)</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -6226,7 +6226,7 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Harriet Bromley (DBZ)</t>
+          <t>Perry Middlebrook (DBZ)</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -6263,17 +6263,17 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Perry Middlebrook (DBZ)</t>
+          <t>Oliver Ashcombe (DBZ)</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Morgan Shaw</t>
+          <t>Parker Jones</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Parker Jones</t>
+          <t>Sam Avery</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -6283,61 +6283,61 @@
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
+          <t>11:30-20:00</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>10:00-18:00</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Wynn Carleton (DBZ)</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Robin Clarke</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Robin Clarke</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>DBZ</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
           <t>07:00-15:30</t>
         </is>
       </c>
-      <c r="F158" s="2" t="inlineStr">
+      <c r="F159" t="inlineStr">
         <is>
           <t>07:00-15:00</t>
         </is>
       </c>
-      <c r="G158" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>Oliver Ashcombe (DBZ)</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
-        <is>
-          <t>Parker Jones</t>
-        </is>
-      </c>
-      <c r="C159" s="2" t="inlineStr">
-        <is>
-          <t>Sam Avery</t>
-        </is>
-      </c>
-      <c r="D159" s="2" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E159" s="2" t="inlineStr">
-        <is>
-          <t>11:30-20:00</t>
-        </is>
-      </c>
-      <c r="F159" s="2" t="inlineStr">
-        <is>
-          <t>10:00-18:00</t>
-        </is>
-      </c>
-      <c r="G159" s="2" t="inlineStr">
-        <is>
-          <t>17</t>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Wynn Carleton (DBZ)</t>
+          <t>Clark Noel (DBZ)</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -6374,7 +6374,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Clark Noel (DBZ)</t>
+          <t>Orin Hartwell (DBZ)</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -6411,7 +6411,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Orin Hartwell (DBZ)</t>
+          <t>Renley Cotsford (DBZ)</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -6448,7 +6448,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Renley Cotsford (DBZ)</t>
+          <t>Nairn Bletchley (DBZ)</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -6485,7 +6485,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Nairn Bletchley (DBZ)</t>
+          <t>Sorrel Beckwith (DBZ)</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -6522,7 +6522,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Sorrel Beckwith (DBZ)</t>
+          <t>Fen Lockhart (DBZ)</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -6559,7 +6559,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Fen Lockhart (DBZ)</t>
+          <t>Piper Matthews (DBZ)</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -6596,7 +6596,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Piper Matthews (DBZ)</t>
+          <t>Teagan Holbrook (DBZ)</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -6633,7 +6633,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Teagan Holbrook (DBZ)</t>
+          <t>Arden Montague (DBZ)</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -6653,7 +6653,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>07:00-15:30</t>
+          <t>13:30-22:00</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -6668,37 +6668,37 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>Arden Montague (DBZ)</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>Carey Westfall (DBZ)</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Morgan</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
         <is>
           <t>Robin Clarke</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>Robin Clarke</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t>13:30-22:00</t>
-        </is>
-      </c>
-      <c r="F169" t="inlineStr">
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>DBZ</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>11:30-20:00</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
         <is>
           <t>07:00-15:00</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr">
+      <c r="G169" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -6707,7 +6707,7 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Carey Westfall (DBZ)</t>
+          <t>Darcy Ellison (DBZ)</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -6742,46 +6742,46 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="inlineStr">
-        <is>
-          <t>Darcy Ellison (DBZ)</t>
-        </is>
-      </c>
-      <c r="B171" s="2" t="inlineStr">
-        <is>
-          <t>Taylor Morgan</t>
-        </is>
-      </c>
-      <c r="C171" s="2" t="inlineStr">
-        <is>
-          <t>Robin Clarke</t>
-        </is>
-      </c>
-      <c r="D171" s="2" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E171" s="2" t="inlineStr">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Hollis Radcliffe (DBZ)</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Rory Sanderson</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Rory Sanderson</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>DBZ</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
         <is>
           <t>11:30-20:00</t>
         </is>
       </c>
-      <c r="F171" s="2" t="inlineStr">
-        <is>
-          <t>07:00-15:00</t>
-        </is>
-      </c>
-      <c r="G171" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>11:30-19:30</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>14</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Hollis Radcliffe (DBZ)</t>
+          <t>Indigo Clarke (DBZ)</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -6818,7 +6818,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Indigo Clarke (DBZ)</t>
+          <t>Eden Beaumont (DBZ)</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -6855,7 +6855,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Eden Beaumont (DBZ)</t>
+          <t>Finley Radcliffe (DBZ)</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -6892,7 +6892,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Finley Radcliffe (DBZ)</t>
+          <t>Winter Grant (DBZ)</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -6929,7 +6929,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Winter Grant (DBZ)</t>
+          <t>Winter Clarke (DBZ)</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -6966,7 +6966,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Winter Clarke (DBZ)</t>
+          <t>Darcy Langley (DBZ)</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -7003,7 +7003,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Darcy Langley (DBZ)</t>
+          <t>Jules Pembroke (DBZ)</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -7040,7 +7040,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Jules Pembroke (DBZ)</t>
+          <t>Addison Fairfax (DBZ)</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -7077,7 +7077,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Addison Fairfax (DBZ)</t>
+          <t>Cameron Hollings (DBZ)</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -7114,7 +7114,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Cameron Hollings (DBZ)</t>
+          <t>Avery Radcliffe (DBZ)</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -7151,7 +7151,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Avery Radcliffe (DBZ)</t>
+          <t>Jordan Walsh (DBZ)</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -7186,46 +7186,46 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>Jordan Walsh (DBZ)</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>Gray Cartwright (DBZ)</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Rory Sanderson</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>Rory Sanderson</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>11:30-20:00</t>
-        </is>
-      </c>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>11:30-19:30</t>
-        </is>
-      </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>14</t>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>Sam Avery</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>DBZ</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>07:00-15:30</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>10:00-18:00</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Gray Cartwright (DBZ)</t>
+          <t>Ellis Beaumont (DBZ)</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -7235,7 +7235,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Sam Avery</t>
+          <t>Jamie Ravenscroft</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -7245,61 +7245,61 @@
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>07:00-15:30</t>
+          <t>08:00-16:30</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>10:00-18:00</t>
+          <t>08:00-16:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="inlineStr">
-        <is>
-          <t>Ellis Beaumont (DBZ)</t>
-        </is>
-      </c>
-      <c r="B185" s="2" t="inlineStr">
-        <is>
-          <t>Rory Sanderson</t>
-        </is>
-      </c>
-      <c r="C185" s="2" t="inlineStr">
-        <is>
-          <t>Jamie Ravenscroft</t>
-        </is>
-      </c>
-      <c r="D185" s="2" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E185" s="2" t="inlineStr">
-        <is>
-          <t>08:00-16:30</t>
-        </is>
-      </c>
-      <c r="F185" s="2" t="inlineStr">
-        <is>
-          <t>08:00-16:00</t>
-        </is>
-      </c>
-      <c r="G185" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Sam Jacobs (DBZ)</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Rowan Carter</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Rowan Carter</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>DBZ</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>11:30-20:00</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>11:30-19:30</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Sam Jacobs (DBZ)</t>
+          <t>Ashton Rowley (DBZ)</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -7336,7 +7336,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Ashton Rowley (DBZ)</t>
+          <t>Skip Jackson (DBZ)</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -7373,7 +7373,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Skip Jackson (DBZ)</t>
+          <t>Perry Walker (DBZ)</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -7410,7 +7410,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Perry Walker (DBZ)</t>
+          <t>Sully Roberts (DBZ)</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -7447,7 +7447,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Sully Roberts (DBZ)</t>
+          <t>Bailey Barrow (DBZ)</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -7484,7 +7484,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Bailey Barrow (DBZ)</t>
+          <t>Sage Edwards (DBZ)</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -7521,7 +7521,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Sage Edwards (DBZ)</t>
+          <t>Cameron Hayes (DBZ)</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -7558,7 +7558,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Cameron Hayes (DBZ)</t>
+          <t>Taylor Birken (DBZ)</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -7595,7 +7595,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Taylor Birken (DBZ)</t>
+          <t>Cameron Alden (DBZ)</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -7632,7 +7632,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Cameron Alden (DBZ)</t>
+          <t>Vivian Burford (DBZ)</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -7652,52 +7652,52 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
+          <t>08:00-16:30</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>11:30-19:30</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Zephyr Langstone (DBZ)</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>Frankie Baxter</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>Rowan Carter</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>DBZ</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
           <t>11:30-20:00</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>11:30-19:30</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>Vivian Burford (DBZ)</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>Rowan Carter</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>Rowan Carter</t>
-        </is>
-      </c>
-      <c r="D196" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>08:00-16:30</t>
-        </is>
-      </c>
-      <c r="F196" t="inlineStr">
-        <is>
-          <t>11:30-19:30</t>
-        </is>
-      </c>
-      <c r="G196" t="inlineStr">
+      <c r="G196" s="2" t="inlineStr">
         <is>
           <t>12</t>
         </is>
@@ -7706,17 +7706,17 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Zephyr Langstone (DBZ)</t>
+          <t>Lane Wetherby (DBZ)</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>Frankie Baxter</t>
+          <t>Sam Avery</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Rowan Carter</t>
+          <t>Hollis Feltham</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
@@ -7726,24 +7726,24 @@
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>11:30-20:00</t>
+          <t>13:30-22:00</t>
         </is>
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>11:30-19:30</t>
+          <t>13:30-22:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Lane Wetherby (DBZ)</t>
+          <t>Merren Southwell (DBZ)</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>Merren Southwell (DBZ)</t>
+          <t>Kerry Larchfield (DBZ)</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Kerry Larchfield (DBZ)</t>
+          <t>Logan Eastman (DBZ)</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -7854,7 +7854,7 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>Logan Eastman (DBZ)</t>
+          <t>Morgan Ashcombe (DBZ)</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -7891,7 +7891,7 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Morgan Ashcombe (DBZ)</t>
+          <t>Ives Blackmore (DBZ)</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -7928,7 +7928,7 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Ives Blackmore (DBZ)</t>
+          <t>Ellis Ravenscroft (DBZ)</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -7965,7 +7965,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Ellis Ravenscroft (DBZ)</t>
+          <t>Rowan Calder (DBZ)</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -8002,7 +8002,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Rowan Calder (DBZ)</t>
+          <t>Hadley Royston (DBZ)</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -8039,12 +8039,12 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Hadley Royston (DBZ)</t>
+          <t>Casey Aldenbrook (DBZ)</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>Sam Avery</t>
+          <t>Morgan Shaw</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
@@ -8076,7 +8076,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Casey Aldenbrook (DBZ)</t>
+          <t>Ember Lewis (DBZ)</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -8113,17 +8113,17 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>Ember Lewis (DBZ)</t>
+          <t>Aubin Harcourt (DBZ)</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>Morgan Shaw</t>
+          <t>Taylor Morgan</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Hollis Feltham</t>
+          <t>Sam Avery</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -8133,24 +8133,24 @@
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>13:30-22:00</t>
+          <t>11:30-20:00</t>
         </is>
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>13:30-22:00</t>
+          <t>10:00-18:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Aubin Harcourt (DBZ)</t>
+          <t>Avery Harrington (DBZ)</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -8187,7 +8187,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Avery Harrington (DBZ)</t>
+          <t>Brook Taverner (DBZ)</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -8224,7 +8224,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Brook Taverner (DBZ)</t>
+          <t>Cassidy Luffman (DBZ)</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -8261,7 +8261,7 @@
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>Cassidy Luffman (DBZ)</t>
+          <t>Harper Blake (DBZ)</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -8298,7 +8298,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>Harper Blake (DBZ)</t>
+          <t>Hayden Burke (DBZ)</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -8335,7 +8335,7 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>Hayden Burke (DBZ)</t>
+          <t>Oakley Jackson (DBZ)</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -8372,7 +8372,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Oakley Jackson (DBZ)</t>
+          <t>Wren Grant (DBZ)</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>11:30-20:00</t>
+          <t>13:30-22:00</t>
         </is>
       </c>
       <c r="F215" s="2" t="inlineStr">
@@ -8409,17 +8409,17 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Wren Grant (DBZ)</t>
+          <t>Bev Stanhope (DBZ)</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>Taylor Morgan</t>
+          <t>Blake Jackson</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Sam Avery</t>
+          <t>Jamie Ravenscroft</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -8429,24 +8429,24 @@
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>13:30-22:00</t>
+          <t>08:00-16:30</t>
         </is>
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>10:00-18:00</t>
+          <t>08:00-16:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Bev Stanhope (DBZ)</t>
+          <t>Bobbie Vickers (DBZ)</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -8483,7 +8483,7 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Bobbie Vickers (DBZ)</t>
+          <t>Ceri Arkwright (DBZ)</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -8520,7 +8520,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Ceri Arkwright (DBZ)</t>
+          <t>Dana Nethercott (DBZ)</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -8557,7 +8557,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Dana Nethercott (DBZ)</t>
+          <t>Dani Newby (DBZ)</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -8594,7 +8594,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Dani Newby (DBZ)</t>
+          <t>Evelyn Yarrow (DBZ)</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -8631,7 +8631,7 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Daryl Loxham (DBZ)</t>
+          <t>Georgie Malleson (DBZ)</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -8668,7 +8668,7 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Evelyn Yarrow (DBZ)</t>
+          <t>Kay Pickering (DBZ)</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -8705,7 +8705,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>Georgie Malleson (DBZ)</t>
+          <t>Kelly Frobisher (DBZ)</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -8742,7 +8742,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Kay Pickering (DBZ)</t>
+          <t>Kim Golding (DBZ)</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -8779,7 +8779,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Kelly Frobisher (DBZ)</t>
+          <t>Leigh Oughton (DBZ)</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -8816,7 +8816,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Kim Golding (DBZ)</t>
+          <t>Loren Peverell (DBZ)</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -8826,7 +8826,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>Jamie Ravenscroft</t>
+          <t>Riley Foster</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -8841,19 +8841,19 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>08:00-16:00</t>
+          <t>14:00-22:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Leigh Oughton (DBZ)</t>
+          <t>Lou Thacker (DBZ)</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Jamie Ravenscroft</t>
+          <t>Riley Foster</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -8878,19 +8878,19 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>08:00-16:00</t>
+          <t>14:00-22:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Loren Peverell (DBZ)</t>
+          <t>Lynn Quenby (DBZ)</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Lou Thacker (DBZ)</t>
+          <t>Marion Gillingham (DBZ)</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -8964,7 +8964,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Lynn Quenby (DBZ)</t>
+          <t>Mel Hargreaves (DBZ)</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -9001,7 +9001,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Marion Gillingham (DBZ)</t>
+          <t>Nicky Dinsmore (DBZ)</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -9038,7 +9038,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Mel Hargreaves (DBZ)</t>
+          <t>Pat Ibbotson (DBZ)</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Nicky Dinsmore (DBZ)</t>
+          <t>Pip Kershaw (DBZ)</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -9112,7 +9112,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Pat Ibbotson (DBZ)</t>
+          <t>Rae Quaife (DBZ)</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -9149,7 +9149,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Pip Kershaw (DBZ)</t>
+          <t>Rene Hepworth (DBZ)</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -9186,7 +9186,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Rae Quaife (DBZ)</t>
+          <t>Ronnie Renshaw (DBZ)</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -9223,7 +9223,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Rene Hepworth (DBZ)</t>
+          <t>Shelley Ingleby (DBZ)</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -9260,7 +9260,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Ronnie Renshaw (DBZ)</t>
+          <t>Stacey Jarvis (DBZ)</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Riley Foster</t>
+          <t>Emerson Clarke</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -9290,14 +9290,14 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Shelley Ingleby (DBZ)</t>
+          <t>Terry Fairbrother (DBZ)</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Riley Foster</t>
+          <t>Emerson Clarke</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -9327,14 +9327,14 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Stacey Jarvis (DBZ)</t>
+          <t>Toni Jowett (DBZ)</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -9371,7 +9371,7 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>Terry Fairbrother (DBZ)</t>
+          <t>Tracy Kingsley (DBZ)</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -9408,7 +9408,7 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Toni Jowett (DBZ)</t>
+          <t>Val Elphick (DBZ)</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -9445,7 +9445,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Tracy Kingsley (DBZ)</t>
+          <t>Vic Sowerby (DBZ)</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -9482,7 +9482,7 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>Val Elphick (DBZ)</t>
+          <t>Jean Ellesmere (DBZ)</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -9502,7 +9502,7 @@
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>08:00-16:30</t>
+          <t>07:00-15:30</t>
         </is>
       </c>
       <c r="F245" s="2" t="inlineStr">
@@ -9519,7 +9519,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>Vic Sowerby (DBZ)</t>
+          <t>Ali Underwood (DBZ)</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>08:00-16:30</t>
+          <t>07:00-15:30</t>
         </is>
       </c>
       <c r="F246" s="2" t="inlineStr">
@@ -9556,7 +9556,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>Jean Ellesmere (DBZ)</t>
+          <t>Jo Chivers (DBZ)</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -9593,7 +9593,7 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>Ali Underwood (DBZ)</t>
+          <t>Jackie Lightfoot (DBZ)</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -9613,7 +9613,7 @@
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>07:00-15:30</t>
+          <t>13:30-22:00</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
@@ -9630,7 +9630,7 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Jo Chivers (DBZ)</t>
+          <t>Gerry Cotswold (DBZ)</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -9650,7 +9650,7 @@
       </c>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>07:00-15:30</t>
+          <t>13:30-22:00</t>
         </is>
       </c>
       <c r="F249" s="2" t="inlineStr">
@@ -9667,7 +9667,7 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Jackie Lightfoot (DBZ)</t>
+          <t>Jan Davenant (DBZ)</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -9687,7 +9687,7 @@
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>13:30-22:00</t>
+          <t>11:30-20:00</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
@@ -9696,80 +9696,6 @@
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" s="2" t="inlineStr">
-        <is>
-          <t>Gerry Cotswold (DBZ)</t>
-        </is>
-      </c>
-      <c r="B251" s="2" t="inlineStr">
-        <is>
-          <t>Blake Jackson</t>
-        </is>
-      </c>
-      <c r="C251" s="2" t="inlineStr">
-        <is>
-          <t>Emerson Clarke</t>
-        </is>
-      </c>
-      <c r="D251" s="2" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E251" s="2" t="inlineStr">
-        <is>
-          <t>13:30-22:00</t>
-        </is>
-      </c>
-      <c r="F251" s="2" t="inlineStr">
-        <is>
-          <t>14:00-22:00</t>
-        </is>
-      </c>
-      <c r="G251" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="2" t="inlineStr">
-        <is>
-          <t>Jan Davenant (DBZ)</t>
-        </is>
-      </c>
-      <c r="B252" s="2" t="inlineStr">
-        <is>
-          <t>Blake Jackson</t>
-        </is>
-      </c>
-      <c r="C252" s="2" t="inlineStr">
-        <is>
-          <t>Emerson Clarke</t>
-        </is>
-      </c>
-      <c r="D252" s="2" t="inlineStr">
-        <is>
-          <t>DBZ</t>
-        </is>
-      </c>
-      <c r="E252" s="2" t="inlineStr">
-        <is>
-          <t>11:30-20:00</t>
-        </is>
-      </c>
-      <c r="F252" s="2" t="inlineStr">
-        <is>
-          <t>14:00-22:00</t>
-        </is>
-      </c>
-      <c r="G252" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>

</xml_diff>